<commit_message>
feat: Task 6 반분 신뢰도 2026 / 2025 (2024 실행 중)
월 안에서 게임 단위 균형 양분, 고정 표면, 선수당 600구로 시즌 간 표본량을
맞추고, 200회 분할 중앙값, 비수축 원값, Spearman-Brown 미보정.

2026: SBJ 0.4929, APR 0.4549, DV_avg 0.4393. 동일 절차로 다시 계산한 ZA는
0.5679다. 기록된 ZA 0.810은 다른 분할과 표본량, 다른 추정 절차의 값이라
새 지표와 직접 비교할 수 없다. 비교 기준은 0.810이 아니라 0.5679다.

2024는 같은 실행에서 계산 중이며 완료 후 별도 커밋. 세 시즌이 모이면 Task 5의
보류된 판정도 함께 정리한다 - DV_avg 신뢰도가 0.44면 잔차 통계량의 블록 간
재현성 0.24 ~ 0.41은 잡음 많은 성분에서 나올 법한 크기다.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JuHKwuzgjEVGuosrkR5rCX
</commit_message>
<xml_diff>
--- a/exports/plate_judgment_2025.xlsx
+++ b/exports/plate_judgment_2025.xlsx
@@ -12,14 +12,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Batters!$A$1:$V$300</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Report!$A$1:$B$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Report!$A$1:$B$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="711">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1158" uniqueCount="736">
   <si>
     <t>season</t>
   </si>
@@ -2152,6 +2152,81 @@
   </si>
   <si>
     <t>["The ABS decision function leaves an asymmetric residual: pitches the rule calls a strike are called balls three to five times more often than the reverse. Unresolved; see ADR-002.", "swing_take._re288 does not shrink, so states seen a handful of times carry an unshrunk run expectancy. See the delta_surface report's re288 block.", "Delta in the Waste region is partly extrapolated and strongly take-favoured; the *_supported_only columns exclude it."]</t>
+  </si>
+  <si>
+    <t>reliability_task6.protocol</t>
+  </si>
+  <si>
+    <t>game-level halves balanced inside each month, fixed surface, 600 pitches per batter per draw, 200 draws, median; raw values, uncorrected</t>
+  </si>
+  <si>
+    <t>reliability_task6.per_batter_sample</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.dv_avg.split_half_r</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.dv_avg.iqr</t>
+  </si>
+  <si>
+    <t>[0.4534, 0.5214]</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.dv_avg.draws</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.dv_avg.median_batters</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.dv_avg.correction</t>
+  </si>
+  <si>
+    <t>none; do not mix with a Spearman-Brown figure</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.apr.split_half_r</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.apr.iqr</t>
+  </si>
+  <si>
+    <t>[0.3626, 0.4471]</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.apr.draws</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.apr.median_batters</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.apr.correction</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.sbj.split_half_r</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.sbj.iqr</t>
+  </si>
+  <si>
+    <t>[0.4281, 0.5064]</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.sbj.draws</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.sbj.median_batters</t>
+  </si>
+  <si>
+    <t>reliability_task6.metrics.sbj.correction</t>
+  </si>
+  <si>
+    <t>reliability_task6.zone_awareness_same_procedure</t>
+  </si>
+  <si>
+    <t>reliability_task6.note</t>
+  </si>
+  <si>
+    <t>ZA's published 0.810 used a different split, sample size and estimator; compare against zone_awareness_same_procedure, not against 0.810</t>
   </si>
 </sst>
 </file>
@@ -22390,7 +22465,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B78"/>
+  <dimension ref="A1:B97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="48.7109375" customWidth="1"/>
@@ -23020,8 +23095,157 @@
         <v>710</v>
       </c>
     </row>
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
+        <v>711</v>
+      </c>
+      <c r="B79" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
+        <v>713</v>
+      </c>
+      <c r="B80">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>714</v>
+      </c>
+      <c r="B81">
+        <v>0.4892</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>715</v>
+      </c>
+      <c r="B82" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" t="s">
+        <v>717</v>
+      </c>
+      <c r="B83">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" t="s">
+        <v>718</v>
+      </c>
+      <c r="B84">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
+        <v>719</v>
+      </c>
+      <c r="B85" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
+        <v>721</v>
+      </c>
+      <c r="B86">
+        <v>0.404</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" t="s">
+        <v>722</v>
+      </c>
+      <c r="B87" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" t="s">
+        <v>724</v>
+      </c>
+      <c r="B88">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
+        <v>725</v>
+      </c>
+      <c r="B89">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
+        <v>726</v>
+      </c>
+      <c r="B90" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>727</v>
+      </c>
+      <c r="B91">
+        <v>0.4754</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>728</v>
+      </c>
+      <c r="B92" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>730</v>
+      </c>
+      <c r="B93">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
+        <v>731</v>
+      </c>
+      <c r="B94">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>732</v>
+      </c>
+      <c r="B95" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
+        <v>734</v>
+      </c>
+      <c r="B97" t="s">
+        <v>735</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B78"/>
+  <autoFilter ref="A1:B97"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>